<commit_message>
Se sube  desarrollo AC12
</commit_message>
<xml_diff>
--- a/LISTA DE FUENTES.xlsx
+++ b/LISTA DE FUENTES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositorio COBOL\COBOL_BATCH_DB2_VSAM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A7E6036-1F49-479E-9E54-EE5034D2DCB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60EC859C-A9AC-4E26-A4A9-B9859F140479}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23064" yWindow="0" windowWidth="23016" windowHeight="12216" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DESARROLLOS" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="130">
   <si>
     <t>PROGRAMA</t>
   </si>
@@ -271,6 +271,138 @@
   </si>
   <si>
     <t>KC02788.ALU9999.COPYLIB(TBVCLIEN)
+KC03C52.CURSOS.DCLGEN(TBCURCLI)</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.FUENTE(EJESIN27)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  TIPO_NOVEDAD; TIPO_DOCUMENTO; NRO_DOCUMENTO; NRO_SECUENCIA
+KEY (1,17)   </t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.FUENTE(JCLDB22)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> BATCH DB2</t>
+  </si>
+  <si>
+    <t>KC03C52.LISTADO.CLIENTES</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.FUENTE(PGMDB022)</t>
+  </si>
+  <si>
+    <t>DB2 SQL\Actividad Actualizar tabla alta o modif - a partir de un txt de novedades\Clase 29 sincrónica - práctica con DB2 _ACT (actualizado).pdf</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.FUENTE(NOVECLIE)</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.FUENTE(JOBDB252)</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.NOVECLIE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FB </t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.FUENTE(PGMDB352)</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.PGMDB352.LISTADO</t>
+  </si>
+  <si>
+    <t>DB2 SQL\Actividad Actualizar tabla alta o modif - a partir de un txt de novedades\EVIDENCIA DE PRUEBA .pdf</t>
+  </si>
+  <si>
+    <t>FUENTES\Corte de control doble _ por tipo documento y genero\Evidencia de prueba_CORTE DE CONTROL DOBLE.pdf</t>
+  </si>
+  <si>
+    <t>FUENTES\Listado con corte de control simple_ por tipo de cuenta\NicoleHeck_Claseasincronica9.pdf</t>
+  </si>
+  <si>
+    <t>FUENTES\RECUPERATORIO PARCIAL I - CORTE DE CONTROL POR TIPO DE CLIENTE\NicoleHeck_EvaluacionCortedeControl.pdf</t>
+  </si>
+  <si>
+    <t>Evaluacion Listado con corte de control simple, por estado civil y acumulacion de importes. Impresion de totales por consola</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.FUENTE(JCORTREC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> KC03C52.CURSOS.FUENTE(PGMREC52)  </t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.CORTE1.SORT</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.FUENTE(CPLAYCOR)</t>
+  </si>
+  <si>
+    <t>tabla DB2 - KC02787.TBCURCTA</t>
+  </si>
+  <si>
+    <t>DB2 SQL\Practica 1 - DB2 SELECT TBCURCTA\Clase 26 sincrónica - práctica con DB2.pdf</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.DCLGEN(TBCURCTA)</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.FUENTE(PGMSIN27)</t>
+  </si>
+  <si>
+    <t>DB2 SQL\Practica INNER JOIN entre tablas con CURSOR y LISTADO\HeckNicole_Claseasincronica11.pdf</t>
+  </si>
+  <si>
+    <t>AC01</t>
+  </si>
+  <si>
+    <t>AC02</t>
+  </si>
+  <si>
+    <t>AC03</t>
+  </si>
+  <si>
+    <t>AC04</t>
+  </si>
+  <si>
+    <t>AC05</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>AC06</t>
+  </si>
+  <si>
+    <t>AC07</t>
+  </si>
+  <si>
+    <t>AC08</t>
+  </si>
+  <si>
+    <t>AC09</t>
+  </si>
+  <si>
+    <t>AC10</t>
+  </si>
+  <si>
+    <t>AC11</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.FUENTE(PGMB5C52)</t>
+  </si>
+  <si>
+    <t>PRC</t>
+  </si>
+  <si>
+    <t>DB2 SQL\PRC_Practica DB2 APAREO - ACTUALIZACION DE SALDOS - Copy\Clase 31 sincrónica - práctica con DB2 apareo ok.pdf</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.FUENTE(NOVCTA)
+KC03C52.CURSOS.DCLGEN(TBCURCTA)
 KC03C52.CURSOS.DCLGEN(TBCURCLI)</t>
   </si>
   <si>
@@ -282,7 +414,7 @@
     <r>
       <rPr>
         <b/>
-        <sz val="11"/>
+        <sz val="12"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
@@ -292,7 +424,7 @@
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
+        <sz val="12"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
@@ -304,135 +436,23 @@
     </r>
   </si>
   <si>
-    <t>KC03C52.CURSOS.FUENTE(EJESIN27)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  TIPO_NOVEDAD; TIPO_DOCUMENTO; NRO_DOCUMENTO; NRO_SECUENCIA
-KEY (1,17)   </t>
-  </si>
-  <si>
-    <t>KC03C52.CURSOS.FUENTE(JCLDB22)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> BATCH DB2</t>
-  </si>
-  <si>
-    <t>KC03C52.LISTADO.CLIENTES</t>
-  </si>
-  <si>
-    <t>KC03C52.CURSOS.FUENTE(PGMDB022)</t>
-  </si>
-  <si>
-    <t>DB2 SQL\Actividad Actualizar tabla alta o modif - a partir de un txt de novedades\Clase 29 sincrónica - práctica con DB2 _ACT (actualizado).pdf</t>
-  </si>
-  <si>
-    <t>KC03C52.CURSOS.FUENTE(NOVECLIE)</t>
-  </si>
-  <si>
-    <t>KC03C52.CURSOS.FUENTE(JOBDB252)</t>
-  </si>
-  <si>
-    <t>KC03C52.CURSOS.NOVECLIE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FB </t>
-  </si>
-  <si>
-    <t>KC03C52.CURSOS.FUENTE(PGMDB352)</t>
-  </si>
-  <si>
-    <t>KC03C52.CURSOS.PGMDB352.LISTADO</t>
-  </si>
-  <si>
-    <t>DB2 SQL\Actividad Actualizar tabla alta o modif - a partir de un txt de novedades\EVIDENCIA DE PRUEBA .pdf</t>
-  </si>
-  <si>
-    <t>FUENTES\Corte de control doble _ por tipo documento y genero\Evidencia de prueba_CORTE DE CONTROL DOBLE.pdf</t>
-  </si>
-  <si>
-    <t>FUENTES\Listado con corte de control simple_ por tipo de cuenta\NicoleHeck_Claseasincronica9.pdf</t>
-  </si>
-  <si>
-    <t>FUENTES\RECUPERATORIO PARCIAL I - CORTE DE CONTROL POR TIPO DE CLIENTE\NicoleHeck_EvaluacionCortedeControl.pdf</t>
-  </si>
-  <si>
-    <t>Evaluacion Listado con corte de control simple, por estado civil y acumulacion de importes. Impresion de totales por consola</t>
-  </si>
-  <si>
-    <t>KC03C52.CURSOS.FUENTE(JCORTREC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> KC03C52.CURSOS.FUENTE(PGMREC52)  </t>
-  </si>
-  <si>
-    <t>KC03C52.CURSOS.CORTE1.SORT</t>
-  </si>
-  <si>
-    <t>KC03C52.CURSOS.FUENTE(CPLAYCOR)</t>
-  </si>
-  <si>
-    <t>tabla DB2 - KC02787.TBCURCTA</t>
-  </si>
-  <si>
-    <t>DB2 SQL\Practica 1 - DB2 SELECT TBCURCTA\Clase 26 sincrónica - práctica con DB2.pdf</t>
-  </si>
-  <si>
-    <t>KC03C52.CURSOS.DCLGEN(TBCURCTA)</t>
-  </si>
-  <si>
-    <t>KC03C52.CURSOS.FUENTE(PGMSIN27)</t>
-  </si>
-  <si>
-    <t>DB2 SQL\Practica INNER JOIN entre tablas con CURSOR y LISTADO\HeckNicole_Claseasincronica11.pdf</t>
-  </si>
-  <si>
-    <t>AC01</t>
-  </si>
-  <si>
-    <t>AC02</t>
-  </si>
-  <si>
-    <t>AC03</t>
-  </si>
-  <si>
-    <t>AC04</t>
-  </si>
-  <si>
-    <t>AC05</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>AC06</t>
-  </si>
-  <si>
-    <t>AC07</t>
-  </si>
-  <si>
-    <t>AC08</t>
-  </si>
-  <si>
-    <t>AC09</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Programa COBOL DB2 con </t>
     </r>
     <r>
       <rPr>
         <b/>
-        <sz val="11"/>
+        <sz val="12"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>cursor</t>
+      <t>CURSOR</t>
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
+        <sz val="12"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
@@ -443,26 +463,41 @@
     </r>
   </si>
   <si>
-    <t>AC10</t>
-  </si>
-  <si>
-    <t>AC11</t>
+    <t>FB</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.FUENTE(JCLDB152)</t>
+  </si>
+  <si>
+    <t>"C:\Users\nicol\Downloads\CODEKI - cobol\DB2 SQL\Practica DB2 APAREO - ACTUALIZACION DE SALDOS - Copy\Logica del programa PGMB5C52.docx"</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.FUENTE(PGMB2C52)</t>
+  </si>
+  <si>
+    <t>KC03C52.ARCHIVO.NOVCTA
+tabla DB2 - KC02787.TBCURCTA
+tabla DB2 - KC02787.TBCURCLI</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.FUENTE(JCLB2C52)</t>
+  </si>
+  <si>
+    <t>AC12</t>
+  </si>
+  <si>
+    <t>DB2 SQL\AC12_Practica Corte de control - SQL COUNT - GROUP BY - ORDER BY\Clase 31   asincrónica 12  - DB2 con CURSOR y CORTE DE CONTROL.pdf</t>
+  </si>
+  <si>
+    <t>DB2 SQL\AC12_Practica Corte de control - SQL COUNT - GROUP BY - ORDER BY\Heck_NicoleDenise_Claseasincronica12.pdf</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -489,8 +524,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -500,12 +558,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -551,77 +603,83 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -954,103 +1012,98 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A2:Q16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" customWidth="1"/>
-    <col min="2" max="2" width="61.42578125" customWidth="1"/>
-    <col min="3" max="3" width="26.85546875" style="3" customWidth="1"/>
-    <col min="4" max="4" width="45" style="8" customWidth="1"/>
-    <col min="5" max="5" width="44.42578125" customWidth="1"/>
-    <col min="6" max="6" width="51.140625" customWidth="1"/>
-    <col min="7" max="7" width="71.7109375" style="20" customWidth="1"/>
-    <col min="8" max="8" width="49.5703125" style="20" customWidth="1"/>
-    <col min="9" max="10" width="14.140625" style="20" customWidth="1"/>
-    <col min="11" max="11" width="16" style="20" customWidth="1"/>
-    <col min="12" max="12" width="34.5703125" style="20" customWidth="1"/>
-    <col min="13" max="13" width="14.140625" style="20" customWidth="1"/>
-    <col min="14" max="14" width="54.7109375" style="3" customWidth="1"/>
-    <col min="15" max="15" width="45" customWidth="1"/>
-    <col min="16" max="16" width="40" style="5" customWidth="1"/>
+    <col min="1" max="1" width="10.28515625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="72.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="26.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="49.85546875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="44.42578125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="51.140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="71.7109375" style="23" customWidth="1"/>
+    <col min="8" max="8" width="49.5703125" style="23" customWidth="1"/>
+    <col min="9" max="10" width="14.140625" style="23" customWidth="1"/>
+    <col min="11" max="11" width="16" style="23" customWidth="1"/>
+    <col min="12" max="12" width="34.5703125" style="23" customWidth="1"/>
+    <col min="13" max="13" width="14.140625" style="23" customWidth="1"/>
+    <col min="14" max="14" width="54.7109375" style="1" customWidth="1"/>
+    <col min="15" max="15" width="45" style="1" customWidth="1"/>
+    <col min="16" max="16" width="40" style="1" customWidth="1"/>
     <col min="17" max="17" width="151.7109375" style="1" customWidth="1"/>
+    <col min="18" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="17"/>
+    <row r="2" spans="1:17" s="7" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="2" spans="1:17" s="3" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="G2" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="I2" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="J2" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="K2" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="L2" s="18" t="s">
-        <v>48</v>
-      </c>
-      <c r="M2" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="O2" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q2" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" s="1" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
+    <row r="3" spans="1:17" s="7" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="7" t="s">
         <v>14</v>
       </c>
       <c r="G3" s="20" t="s">
@@ -1074,36 +1127,36 @@
       <c r="M3" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="N3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="O3" s="1" t="s">
+      <c r="O3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="P3" s="3">
+      <c r="P3" s="7">
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:17" s="1" customFormat="1" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="B4" s="1" t="s">
+    <row r="4" spans="1:17" s="7" customFormat="1" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="21" t="s">
+      <c r="G4" s="19" t="s">
         <v>9</v>
       </c>
       <c r="H4" s="20" t="s">
@@ -1124,36 +1177,36 @@
       <c r="M4" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="N4" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="O4" s="1" t="s">
+      <c r="O4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="P4" s="3">
+      <c r="P4" s="7">
         <v>30</v>
       </c>
-      <c r="Q4" s="6" t="s">
+      <c r="Q4" s="11" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:17" s="1" customFormat="1" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="B5" s="1" t="s">
+    <row r="5" spans="1:17" s="7" customFormat="1" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="7" t="s">
         <v>2</v>
       </c>
       <c r="G5" s="20" t="s">
@@ -1177,36 +1230,36 @@
       <c r="M5" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="N5" s="3" t="s">
+      <c r="N5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="O5" s="1" t="s">
+      <c r="O5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="P5" s="3">
+      <c r="P5" s="7">
         <v>93</v>
       </c>
-      <c r="Q5" s="7" t="s">
+      <c r="Q5" s="12" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:17" s="1" customFormat="1" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="B6" s="1" t="s">
+    <row r="6" spans="1:17" s="7" customFormat="1" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="7" t="s">
         <v>42</v>
       </c>
       <c r="G6" s="20" t="s">
@@ -1230,36 +1283,36 @@
       <c r="M6" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="N6" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="O6" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P6" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q6" s="7" t="s">
-        <v>92</v>
+      <c r="N6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="P6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q6" s="12" t="s">
+        <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:17" s="1" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="B7" s="1" t="s">
+    <row r="7" spans="1:17" s="7" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="23" t="s">
+      <c r="C7" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="7" t="s">
         <v>29</v>
       </c>
       <c r="G7" s="20" t="s">
@@ -1283,36 +1336,36 @@
       <c r="M7" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="N7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="O7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q7" s="7" t="s">
-        <v>91</v>
+      <c r="N7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="O7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="P7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q7" s="12" t="s">
+        <v>90</v>
       </c>
     </row>
-    <row r="8" spans="1:17" s="1" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="B8" s="1" t="s">
+    <row r="8" spans="1:17" s="7" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="7" t="s">
         <v>35</v>
       </c>
       <c r="G8" s="20" t="s">
@@ -1336,43 +1389,43 @@
       <c r="M8" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="N8" s="3" t="s">
+      <c r="N8" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="O8" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P8" s="3">
+      <c r="O8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="P8" s="7">
         <v>133</v>
       </c>
-      <c r="Q8" s="7" t="s">
+      <c r="Q8" s="12" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:17" s="1" customFormat="1" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="B9" s="2" t="s">
+    <row r="9" spans="1:17" s="7" customFormat="1" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E9" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G9" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="G9" s="20" t="s">
+      <c r="H9" s="20" t="s">
         <v>97</v>
-      </c>
-      <c r="H9" s="20" t="s">
-        <v>98</v>
       </c>
       <c r="I9" s="20">
         <v>126</v>
@@ -1389,127 +1442,132 @@
       <c r="M9" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="N9" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="O9" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P9" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q9" s="7" t="s">
-        <v>93</v>
+      <c r="N9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="O9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="P9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q9" s="12" t="s">
+        <v>92</v>
       </c>
     </row>
-    <row r="10" spans="1:17" s="1" customFormat="1" ht="138" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="B10" s="2" t="s">
+    <row r="10" spans="1:17" s="7" customFormat="1" ht="138" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G10" s="21" t="s">
+      <c r="G10" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="H10" s="21" t="s">
+      <c r="H10" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="I10" s="21" t="s">
+      <c r="I10" s="19" t="s">
         <v>50</v>
       </c>
       <c r="J10" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="K10" s="21" t="s">
+      <c r="K10" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="L10" s="21" t="s">
+      <c r="L10" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="M10" s="21" t="s">
+      <c r="M10" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="N10" s="3" t="s">
+      <c r="N10" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="O10" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P10" s="3">
+      <c r="O10" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="P10" s="7">
         <v>133</v>
       </c>
-      <c r="Q10" s="10" t="s">
+      <c r="Q10" s="13" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="174.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:17" s="7" customFormat="1" ht="174.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="G11" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="H11" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="I11" s="20"/>
+      <c r="J11" s="20"/>
+      <c r="K11" s="20"/>
+      <c r="L11" s="20"/>
+      <c r="M11" s="20"/>
+      <c r="N11" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q11" s="12" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" s="7" customFormat="1" ht="203.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="B11" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="D11" s="11" t="s">
+      <c r="B12" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D12" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G11" s="20" t="s">
-        <v>99</v>
-      </c>
-      <c r="H11" s="20" t="s">
+      <c r="E12" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F12" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="N11" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q11" s="7" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" ht="203.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="G12" s="21" t="s">
+      <c r="G12" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="H12" s="21" t="s">
+      <c r="H12" s="19" t="s">
         <v>75</v>
       </c>
       <c r="I12" s="20">
@@ -1521,105 +1579,105 @@
       <c r="K12" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="L12" s="21" t="s">
+      <c r="L12" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="M12" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="N12" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="O12" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="P12" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" s="7" customFormat="1" ht="87" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E13" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="M12" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="N12" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="O12" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P12" s="3" t="s">
-        <v>33</v>
+      <c r="F13" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="G13" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="H13" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="I13" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="J13" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="K13" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="L13" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="M13" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="N13" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="O13" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="P13" s="7">
+        <v>133</v>
+      </c>
+      <c r="Q13" s="12" t="s">
+        <v>102</v>
       </c>
     </row>
-    <row r="13" spans="1:17" ht="87" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="B13" s="2" t="s">
+    <row r="14" spans="1:17" s="7" customFormat="1" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D13" s="11" t="s">
+      <c r="B14" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D14" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="G13" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="H13" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="I13" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="J13" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="K13" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="L13" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="M13" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="N13" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="O13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P13" s="3">
-        <v>133</v>
-      </c>
-      <c r="Q13" s="15" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" ht="120" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="B14" s="10" t="s">
+      <c r="E14" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="G14" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="H14" s="20" t="s">
         <v>83</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="F14" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="G14" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="H14" s="20" t="s">
-        <v>84</v>
       </c>
       <c r="I14" s="20">
         <v>80</v>
       </c>
       <c r="J14" s="20" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="K14" s="20" t="s">
         <v>46</v>
@@ -1627,21 +1685,122 @@
       <c r="L14" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="N14" s="16" t="s">
+      <c r="M14" s="20"/>
+      <c r="N14" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="O14" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="P14" s="7">
+        <v>133</v>
+      </c>
+      <c r="Q14" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="O14" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P14" s="3">
-        <v>133</v>
-      </c>
-      <c r="Q14" s="7" t="s">
-        <v>90</v>
+    </row>
+    <row r="15" spans="1:17" s="16" customFormat="1" ht="134.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="B15" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="G15" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="H15" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="I15" s="20">
+        <v>23</v>
+      </c>
+      <c r="J15" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="K15" s="20"/>
+      <c r="L15" s="20"/>
+      <c r="M15" s="20"/>
+      <c r="N15" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="O15" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="P15" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q15" s="21" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" s="22" customFormat="1" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="B16" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="E16" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="F16" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="G16" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="H16" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="I16" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="J16" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="K16" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="L16" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="M16" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="N16" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="O16" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="P16" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q16" s="21" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="Q4" r:id="rId1" xr:uid="{204D8A35-8951-4CCB-8A53-F0ACD5058904}"/>
     <hyperlink ref="Q5" r:id="rId2" xr:uid="{C5784AB5-52E9-4628-AD2B-EF82847E2338}"/>
@@ -1654,9 +1813,13 @@
     <hyperlink ref="Q9" r:id="rId9" xr:uid="{2040CF26-0E2F-4E22-AAFD-5CA719469C7E}"/>
     <hyperlink ref="Q11" r:id="rId10" xr:uid="{A40DE3A8-D393-4C3C-80BE-F5E084F7D368}"/>
     <hyperlink ref="Q13" r:id="rId11" xr:uid="{DC1A933C-9A6F-4C74-AED3-249F8FF69FA7}"/>
+    <hyperlink ref="B15" r:id="rId12" xr:uid="{C393B9C1-2534-4D46-BC85-EFF04E89A099}"/>
+    <hyperlink ref="Q15" r:id="rId13" xr:uid="{CC6455DB-4674-4CAE-9E56-BE1779B5BF37}"/>
+    <hyperlink ref="B16" r:id="rId14" xr:uid="{AE230BC1-C26C-489D-84B5-A4401AC05727}"/>
+    <hyperlink ref="Q16" r:id="rId15" xr:uid="{AE550FB3-F106-4DC4-BCB8-8DAFC8F47C9B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId12"/>
-  <drawing r:id="rId13"/>
+  <pageSetup orientation="portrait" r:id="rId16"/>
+  <drawing r:id="rId17"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Se sube PRC2 y MODEXAMEN1
</commit_message>
<xml_diff>
--- a/LISTA DE FUENTES.xlsx
+++ b/LISTA DE FUENTES.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositorio COBOL\COBOL_BATCH_DB2_VSAM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60EC859C-A9AC-4E26-A4A9-B9859F140479}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF74982D-2169-4834-8BE9-1A5F65DB2FAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="23064" yWindow="0" windowWidth="23016" windowHeight="12216" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="149">
   <si>
     <t>PROGRAMA</t>
   </si>
@@ -393,9 +393,6 @@
   </si>
   <si>
     <t>KC03C52.CURSOS.FUENTE(PGMB5C52)</t>
-  </si>
-  <si>
-    <t>PRC</t>
   </si>
   <si>
     <t>DB2 SQL\PRC_Practica DB2 APAREO - ACTUALIZACION DE SALDOS - Copy\Clase 31 sincrónica - práctica con DB2 apareo ok.pdf</t>
@@ -490,6 +487,68 @@
   </si>
   <si>
     <t>DB2 SQL\AC12_Practica Corte de control - SQL COUNT - GROUP BY - ORDER BY\Heck_NicoleDenise_Claseasincronica12.pdf</t>
+  </si>
+  <si>
+    <t>PRC2</t>
+  </si>
+  <si>
+    <t>PRC1</t>
+  </si>
+  <si>
+    <t>KC03C52.LISTADO.CONTROL</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.DCLGEN(TBCURCTA)
+KC03C52.CURSOS.DCLGEN(TBCURCLI)</t>
+  </si>
+  <si>
+    <t>tabla DB2 - KC02787.TBCURCTA
+tabla DB2 - KC02787.TBCURCLI</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.FUENTE(PGMV2C52)</t>
+  </si>
+  <si>
+    <t>DB2 SQL\PRC2_Clase 33 Sincronica -  Control de integridad y duplicidades (DB2 + COBOL)\Clase 33 Sincronica -  Control de integridad y duplicidades (DB2 + COBOL).pdf</t>
+  </si>
+  <si>
+    <t>PRC0</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.FUENTE(JCLV2C52)</t>
+  </si>
+  <si>
+    <t>DB2 SQL\PRC2_Clase 33 Sincronica -  Control de integridad y duplicidades (DB2 + COBOL)\EVIDENCIA DE PRUEBA.pdf</t>
+  </si>
+  <si>
+    <t>JEXAMEN1</t>
+  </si>
+  <si>
+    <t>EXAMEN1</t>
+  </si>
+  <si>
+    <t>KC03C52.ARCHIVO.NOVCTA</t>
+  </si>
+  <si>
+    <t>KC03C52.CURSOS.FUENTE(NOVCTA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Este programaLEE NOVCTA, realiza un CORTE DE CONTROL DOBLE. Trabaja con CURSOR, accede a tabla TBCURCTA y graba un listado. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Este programa LEE NOVECLI,  realiza un CORTE DE CONTROL DOBLE. Trabaja con CURSOR, accede a tabla TBCURCLI y graba un listado. </t>
+  </si>
+  <si>
+    <t>MODEXAMEN1</t>
+  </si>
+  <si>
+    <t>MODEXAMEN2</t>
+  </si>
+  <si>
+    <t>EXAMEN2</t>
+  </si>
+  <si>
+    <t>JEXAMEN2</t>
   </si>
 </sst>
 </file>
@@ -605,7 +664,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -652,35 +711,32 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1012,21 +1068,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:Q16"/>
+  <dimension ref="A2:Q20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="72.28515625" style="1" customWidth="1"/>
     <col min="3" max="3" width="26.85546875" style="1" customWidth="1"/>
     <col min="4" max="4" width="49.85546875" style="2" customWidth="1"/>
     <col min="5" max="5" width="44.42578125" style="1" customWidth="1"/>
     <col min="6" max="6" width="51.140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="71.7109375" style="23" customWidth="1"/>
-    <col min="8" max="8" width="49.5703125" style="23" customWidth="1"/>
-    <col min="9" max="10" width="14.140625" style="23" customWidth="1"/>
-    <col min="11" max="11" width="16" style="23" customWidth="1"/>
-    <col min="12" max="12" width="34.5703125" style="23" customWidth="1"/>
-    <col min="13" max="13" width="14.140625" style="23" customWidth="1"/>
+    <col min="7" max="7" width="71.7109375" style="20" customWidth="1"/>
+    <col min="8" max="8" width="49.5703125" style="20" customWidth="1"/>
+    <col min="9" max="10" width="14.140625" style="20" customWidth="1"/>
+    <col min="11" max="11" width="16" style="20" customWidth="1"/>
+    <col min="12" max="12" width="34.5703125" style="20" customWidth="1"/>
+    <col min="13" max="13" width="14.140625" style="20" customWidth="1"/>
     <col min="14" max="14" width="54.7109375" style="1" customWidth="1"/>
     <col min="15" max="15" width="45" style="1" customWidth="1"/>
     <col min="16" max="16" width="40" style="1" customWidth="1"/>
@@ -1089,7 +1145,7 @@
     </row>
     <row r="3" spans="1:17" s="7" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>116</v>
+        <v>136</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>23</v>
@@ -1106,25 +1162,25 @@
       <c r="F3" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G3" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="20" t="s">
+      <c r="H3" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="I3" s="20">
+      <c r="I3" s="18">
         <v>50</v>
       </c>
-      <c r="J3" s="20" t="s">
+      <c r="J3" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="K3" s="20" t="s">
+      <c r="K3" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="L3" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="M3" s="20" t="s">
+      <c r="L3" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="M3" s="18" t="s">
         <v>33</v>
       </c>
       <c r="N3" s="7" t="s">
@@ -1156,25 +1212,25 @@
       <c r="F4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="20" t="s">
+      <c r="H4" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="20">
+      <c r="I4" s="18">
         <v>30</v>
       </c>
-      <c r="J4" s="20" t="s">
+      <c r="J4" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="K4" s="20" t="s">
+      <c r="K4" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="L4" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="M4" s="20" t="s">
+      <c r="L4" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="M4" s="18" t="s">
         <v>33</v>
       </c>
       <c r="N4" s="7" t="s">
@@ -1209,25 +1265,25 @@
       <c r="F5" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="G5" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="20" t="s">
+      <c r="H5" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="20">
+      <c r="I5" s="18">
         <v>93</v>
       </c>
-      <c r="J5" s="20" t="s">
+      <c r="J5" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="K5" s="20" t="s">
+      <c r="K5" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="L5" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="M5" s="20" t="s">
+      <c r="L5" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="M5" s="18" t="s">
         <v>33</v>
       </c>
       <c r="N5" s="7" t="s">
@@ -1262,25 +1318,25 @@
       <c r="F6" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="G6" s="20" t="s">
+      <c r="G6" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="20" t="s">
+      <c r="H6" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="I6" s="20">
+      <c r="I6" s="18">
         <v>93</v>
       </c>
-      <c r="J6" s="20" t="s">
+      <c r="J6" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="K6" s="20" t="s">
+      <c r="K6" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="L6" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="M6" s="20" t="s">
+      <c r="L6" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="M6" s="18" t="s">
         <v>33</v>
       </c>
       <c r="N6" s="7" t="s">
@@ -1315,25 +1371,25 @@
       <c r="F7" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="20" t="s">
+      <c r="G7" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="20" t="s">
+      <c r="H7" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="20">
+      <c r="I7" s="18">
         <v>93</v>
       </c>
-      <c r="J7" s="20" t="s">
+      <c r="J7" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="K7" s="20" t="s">
+      <c r="K7" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="L7" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="M7" s="20" t="s">
+      <c r="L7" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="M7" s="18" t="s">
         <v>33</v>
       </c>
       <c r="N7" s="7" t="s">
@@ -1368,25 +1424,25 @@
       <c r="F8" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="G8" s="20" t="s">
+      <c r="G8" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="H8" s="20" t="s">
+      <c r="H8" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="I8" s="20">
+      <c r="I8" s="18">
         <v>50</v>
       </c>
-      <c r="J8" s="20" t="s">
+      <c r="J8" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="K8" s="20" t="s">
+      <c r="K8" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="L8" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="M8" s="20" t="s">
+      <c r="L8" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="M8" s="18" t="s">
         <v>33</v>
       </c>
       <c r="N8" s="7" t="s">
@@ -1421,25 +1477,25 @@
       <c r="F9" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="G9" s="20" t="s">
+      <c r="G9" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="H9" s="20" t="s">
+      <c r="H9" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="I9" s="20">
+      <c r="I9" s="18">
         <v>126</v>
       </c>
-      <c r="J9" s="20" t="s">
+      <c r="J9" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="K9" s="20" t="s">
+      <c r="K9" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="L9" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="M9" s="20" t="s">
+      <c r="L9" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="M9" s="18" t="s">
         <v>33</v>
       </c>
       <c r="N9" s="7" t="s">
@@ -1455,7 +1511,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="10" spans="1:17" s="7" customFormat="1" ht="138" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" s="7" customFormat="1" ht="186.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>110</v>
       </c>
@@ -1474,25 +1530,25 @@
       <c r="F10" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G10" s="19" t="s">
+      <c r="G10" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="H10" s="19" t="s">
+      <c r="H10" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="I10" s="19" t="s">
+      <c r="I10" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="J10" s="20" t="s">
+      <c r="J10" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="K10" s="19" t="s">
+      <c r="K10" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="L10" s="19" t="s">
+      <c r="L10" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="M10" s="19" t="s">
+      <c r="M10" s="17" t="s">
         <v>54</v>
       </c>
       <c r="N10" s="7" t="s">
@@ -1527,17 +1583,17 @@
       <c r="F11" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="G11" s="20" t="s">
+      <c r="G11" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="H11" s="20" t="s">
+      <c r="H11" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="I11" s="20"/>
-      <c r="J11" s="20"/>
-      <c r="K11" s="20"/>
-      <c r="L11" s="20"/>
-      <c r="M11" s="20"/>
+      <c r="I11" s="18"/>
+      <c r="J11" s="18"/>
+      <c r="K11" s="18"/>
+      <c r="L11" s="18"/>
+      <c r="M11" s="18"/>
       <c r="N11" s="7" t="s">
         <v>71</v>
       </c>
@@ -1550,7 +1606,7 @@
         <v>112</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>72</v>
@@ -1564,25 +1620,25 @@
       <c r="F12" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="G12" s="19" t="s">
+      <c r="G12" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="H12" s="19" t="s">
+      <c r="H12" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="I12" s="20">
+      <c r="I12" s="18">
         <v>244</v>
       </c>
-      <c r="J12" s="20" t="s">
+      <c r="J12" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="K12" s="20" t="s">
+      <c r="K12" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="L12" s="19" t="s">
+      <c r="L12" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="M12" s="20" t="s">
+      <c r="M12" s="18" t="s">
         <v>33</v>
       </c>
       <c r="N12" s="7" t="s">
@@ -1600,7 +1656,7 @@
         <v>113</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>79</v>
@@ -1614,25 +1670,25 @@
       <c r="F13" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="G13" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="H13" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="I13" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="J13" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="K13" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="L13" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="M13" s="20" t="s">
+      <c r="G13" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="H13" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="I13" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="J13" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="K13" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="L13" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="M13" s="18" t="s">
         <v>33</v>
       </c>
       <c r="N13" s="7" t="s">
@@ -1667,25 +1723,25 @@
       <c r="F14" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="G14" s="25" t="s">
+      <c r="G14" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="H14" s="20" t="s">
+      <c r="H14" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="I14" s="20">
+      <c r="I14" s="18">
         <v>80</v>
       </c>
-      <c r="J14" s="20" t="s">
+      <c r="J14" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="K14" s="20" t="s">
+      <c r="K14" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="L14" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="M14" s="20"/>
+      <c r="L14" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="M14" s="18"/>
       <c r="N14" s="15" t="s">
         <v>88</v>
       </c>
@@ -1699,105 +1755,214 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:17" s="16" customFormat="1" ht="134.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="16" t="s">
+    <row r="15" spans="1:17" s="7" customFormat="1" ht="134.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B15" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="C15" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="G15" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="H15" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="I15" s="18">
+        <v>23</v>
+      </c>
+      <c r="J15" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="K15" s="18"/>
+      <c r="L15" s="18"/>
+      <c r="M15" s="18"/>
+      <c r="N15" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="O15" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="P15" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q15" s="19" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="B16" s="21" t="s">
+        <v>127</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D15" s="18" t="s">
+      <c r="D16" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="16" t="s">
-        <v>122</v>
-      </c>
-      <c r="F15" s="16" t="s">
-        <v>115</v>
-      </c>
-      <c r="G15" s="19" t="s">
+      <c r="E16" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="H15" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="I15" s="20">
-        <v>23</v>
-      </c>
-      <c r="J15" s="20" t="s">
-        <v>121</v>
-      </c>
-      <c r="K15" s="20"/>
-      <c r="L15" s="20"/>
-      <c r="M15" s="20"/>
-      <c r="N15" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="O15" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="P15" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q15" s="21" t="s">
+      <c r="F16" s="1" t="s">
         <v>123</v>
       </c>
+      <c r="G16" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="H16" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="I16" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="J16" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="K16" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="L16" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="M16" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="N16" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="O16" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="P16" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q16" s="19" t="s">
+        <v>128</v>
+      </c>
     </row>
-    <row r="16" spans="1:17" s="22" customFormat="1" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="22" t="s">
-        <v>127</v>
-      </c>
-      <c r="B16" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="C16" s="16" t="s">
+    <row r="17" spans="1:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B17" s="21" t="s">
+        <v>135</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="D17" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="E16" s="22" t="s">
-        <v>126</v>
-      </c>
-      <c r="F16" s="22" t="s">
-        <v>124</v>
-      </c>
-      <c r="G16" s="20" t="s">
-        <v>98</v>
-      </c>
-      <c r="H16" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="I16" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="J16" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="K16" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="L16" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="M16" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="N16" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="O16" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="P16" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q16" s="21" t="s">
-        <v>129</v>
-      </c>
+      <c r="E17" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="G17" s="17" t="s">
+        <v>133</v>
+      </c>
+      <c r="H17" s="24" t="s">
+        <v>132</v>
+      </c>
+      <c r="I17" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="J17" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="K17" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="L17" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="M17" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="N17" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="O17" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="P17" s="7">
+        <v>133</v>
+      </c>
+      <c r="Q17" s="19" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="B18" s="23" t="s">
+        <v>144</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="G18" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="H18" s="18" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="B19" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="G19" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="H19" s="18" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C20" s="7"/>
+      <c r="D20" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1817,9 +1982,11 @@
     <hyperlink ref="Q15" r:id="rId13" xr:uid="{CC6455DB-4674-4CAE-9E56-BE1779B5BF37}"/>
     <hyperlink ref="B16" r:id="rId14" xr:uid="{AE230BC1-C26C-489D-84B5-A4401AC05727}"/>
     <hyperlink ref="Q16" r:id="rId15" xr:uid="{AE550FB3-F106-4DC4-BCB8-8DAFC8F47C9B}"/>
+    <hyperlink ref="B17" r:id="rId16" xr:uid="{628BD9B7-9D4C-4B3C-8C6D-EB3C5AD5CDD8}"/>
+    <hyperlink ref="Q17" r:id="rId17" xr:uid="{06171273-33A9-406B-86DE-A35C80604BBA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId16"/>
-  <drawing r:id="rId17"/>
+  <pageSetup orientation="portrait" r:id="rId18"/>
+  <drawing r:id="rId19"/>
 </worksheet>
 </file>
</xml_diff>